<commit_message>
arregle excel y coloque nuevaente las tarjetas como estaban
</commit_message>
<xml_diff>
--- a/assets/plantillas/Registro de Radicación de Comunicaciones Oficiales Salientes.xlsx
+++ b/assets/plantillas/Registro de Radicación de Comunicaciones Oficiales Salientes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\OSCAR\Documents\VENTANILLA UNICA DE CORRESPONDENCIA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A52F2F09-BBAC-431C-9D5D-605B59A44A06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7917988-FD4E-449F-9837-2B6CC7336F70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="531" xr2:uid="{01888BE3-A2F9-459F-9A94-C37BE0E28B96}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="531" xr2:uid="{01888BE3-A2F9-459F-9A94-C37BE0E28B96}"/>
   </bookViews>
   <sheets>
     <sheet name="F03" sheetId="1" r:id="rId1"/>
@@ -236,7 +236,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -304,10 +304,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -788,59 +784,59 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B32D33D-A55A-45BC-BAAA-C6712B8A707F}">
   <dimension ref="A1:I237"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="0" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="0" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.5703125" style="4" customWidth="1"/>
-    <col min="2" max="2" width="17.7109375" style="8" customWidth="1"/>
-    <col min="3" max="3" width="16.5703125" style="8" customWidth="1"/>
-    <col min="4" max="4" width="32.28515625" style="4" customWidth="1"/>
-    <col min="5" max="5" width="54.7109375" style="4" customWidth="1"/>
-    <col min="6" max="7" width="9.7109375" style="4" customWidth="1"/>
-    <col min="8" max="8" width="18.7109375" style="4" customWidth="1"/>
-    <col min="9" max="9" width="33.85546875" style="4" customWidth="1"/>
-    <col min="10" max="10" width="3.42578125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="17.5546875" style="4" customWidth="1"/>
+    <col min="2" max="2" width="17.6640625" style="8" customWidth="1"/>
+    <col min="3" max="3" width="16.5546875" style="8" customWidth="1"/>
+    <col min="4" max="4" width="32.33203125" style="4" customWidth="1"/>
+    <col min="5" max="5" width="54.6640625" style="4" customWidth="1"/>
+    <col min="6" max="7" width="9.6640625" style="4" customWidth="1"/>
+    <col min="8" max="8" width="18.6640625" style="4" customWidth="1"/>
+    <col min="9" max="9" width="33.88671875" style="4" customWidth="1"/>
+    <col min="10" max="10" width="3.44140625" style="1" customWidth="1"/>
     <col min="11" max="16384" width="0" style="1" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="7.5" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A2" s="22"/>
-      <c r="B2" s="23" t="s">
+    <row r="1" spans="1:9" ht="7.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="21"/>
+      <c r="B2" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="23"/>
-      <c r="H2" s="24" t="s">
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="I2" s="22" t="s">
+      <c r="I2" s="21" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A3" s="22"/>
-      <c r="B3" s="23"/>
-      <c r="C3" s="23"/>
-      <c r="D3" s="23"/>
-      <c r="E3" s="23"/>
-      <c r="F3" s="23"/>
-      <c r="G3" s="23"/>
-      <c r="H3" s="24"/>
-      <c r="I3" s="22"/>
-    </row>
-    <row r="4" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="22"/>
-      <c r="B4" s="23" t="s">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="21"/>
+      <c r="B3" s="22"/>
+      <c r="C3" s="22"/>
+      <c r="D3" s="22"/>
+      <c r="E3" s="22"/>
+      <c r="F3" s="22"/>
+      <c r="G3" s="22"/>
+      <c r="H3" s="23"/>
+      <c r="I3" s="21"/>
+    </row>
+    <row r="4" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="21"/>
+      <c r="B4" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="23"/>
-      <c r="D4" s="23"/>
-      <c r="E4" s="23"/>
-      <c r="F4" s="23"/>
-      <c r="G4" s="23"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
+      <c r="G4" s="22"/>
       <c r="H4" s="2" t="s">
         <v>1</v>
       </c>
@@ -848,14 +844,14 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="15" x14ac:dyDescent="0.2">
-      <c r="A5" s="22"/>
-      <c r="B5" s="23"/>
-      <c r="C5" s="23"/>
-      <c r="D5" s="23"/>
-      <c r="E5" s="23"/>
-      <c r="F5" s="23"/>
-      <c r="G5" s="23"/>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="21"/>
+      <c r="B5" s="22"/>
+      <c r="C5" s="22"/>
+      <c r="D5" s="22"/>
+      <c r="E5" s="22"/>
+      <c r="F5" s="22"/>
+      <c r="G5" s="22"/>
       <c r="H5" s="2" t="s">
         <v>2</v>
       </c>
@@ -863,20 +859,20 @@
         <v>45656</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="25" t="s">
+    <row r="6" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="25"/>
-      <c r="C6" s="26"/>
-      <c r="D6" s="26"/>
-      <c r="E6" s="26"/>
-      <c r="F6" s="26"/>
-      <c r="G6" s="26"/>
-      <c r="H6" s="26"/>
-      <c r="I6" s="27"/>
-    </row>
-    <row r="7" spans="1:9" s="3" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="B6" s="24"/>
+      <c r="C6" s="25"/>
+      <c r="D6" s="25"/>
+      <c r="E6" s="25"/>
+      <c r="F6" s="25"/>
+      <c r="G6" s="25"/>
+      <c r="H6" s="25"/>
+      <c r="I6" s="26"/>
+    </row>
+    <row r="7" spans="1:9" s="3" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
         <v>7</v>
       </c>
@@ -905,7 +901,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:9" s="4" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:9" s="4" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>15</v>
       </c>
@@ -920,7 +916,7 @@
       <c r="H8" s="14"/>
       <c r="I8" s="12"/>
     </row>
-    <row r="9" spans="1:9" s="4" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:9" s="4" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
         <v>16</v>
       </c>
@@ -933,7 +929,7 @@
       <c r="H9" s="14"/>
       <c r="I9" s="12"/>
     </row>
-    <row r="10" spans="1:9" s="4" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:9" s="4" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
         <v>17</v>
       </c>
@@ -946,7 +942,7 @@
       <c r="H10" s="14"/>
       <c r="I10" s="12"/>
     </row>
-    <row r="11" spans="1:9" s="4" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:9" s="4" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>18</v>
       </c>
@@ -959,7 +955,7 @@
       <c r="H11" s="14"/>
       <c r="I11" s="12"/>
     </row>
-    <row r="12" spans="1:9" s="4" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:9" s="4" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
         <v>19</v>
       </c>
@@ -972,7 +968,7 @@
       <c r="H12" s="14"/>
       <c r="I12" s="12"/>
     </row>
-    <row r="13" spans="1:9" s="4" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:9" s="4" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
         <v>20</v>
       </c>
@@ -985,7 +981,7 @@
       <c r="H13" s="12"/>
       <c r="I13" s="12"/>
     </row>
-    <row r="14" spans="1:9" s="4" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:9" s="4" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
         <v>21</v>
       </c>
@@ -998,7 +994,7 @@
       <c r="H14" s="12"/>
       <c r="I14" s="12"/>
     </row>
-    <row r="15" spans="1:9" s="4" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:9" s="4" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
         <v>22</v>
       </c>
@@ -1011,7 +1007,7 @@
       <c r="H15" s="12"/>
       <c r="I15" s="12"/>
     </row>
-    <row r="16" spans="1:9" s="4" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:9" s="4" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
         <v>23</v>
       </c>
@@ -1024,7 +1020,7 @@
       <c r="H16" s="12"/>
       <c r="I16" s="12"/>
     </row>
-    <row r="17" spans="1:9" s="4" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:9" s="4" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
         <v>24</v>
       </c>
@@ -1037,7 +1033,7 @@
       <c r="H17" s="16"/>
       <c r="I17" s="12"/>
     </row>
-    <row r="18" spans="1:9" s="4" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:9" s="4" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="12"/>
       <c r="B18" s="9"/>
       <c r="C18" s="9"/>
@@ -1048,7 +1044,7 @@
       <c r="H18" s="16"/>
       <c r="I18" s="12"/>
     </row>
-    <row r="19" spans="1:9" s="4" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:9" s="4" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="12"/>
       <c r="B19" s="9"/>
       <c r="C19" s="9"/>
@@ -1059,7 +1055,7 @@
       <c r="H19" s="16"/>
       <c r="I19" s="12"/>
     </row>
-    <row r="20" spans="1:9" s="4" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:9" s="4" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="12"/>
       <c r="B20" s="9"/>
       <c r="C20" s="9"/>
@@ -1070,7 +1066,7 @@
       <c r="H20" s="16"/>
       <c r="I20" s="12"/>
     </row>
-    <row r="21" spans="1:9" s="4" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:9" s="4" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="12"/>
       <c r="B21" s="9"/>
       <c r="C21" s="9"/>
@@ -1081,7 +1077,7 @@
       <c r="H21" s="16"/>
       <c r="I21" s="14"/>
     </row>
-    <row r="22" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="12"/>
       <c r="B22" s="9"/>
       <c r="C22" s="9"/>
@@ -1092,7 +1088,7 @@
       <c r="H22" s="16"/>
       <c r="I22" s="16"/>
     </row>
-    <row r="23" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="12"/>
       <c r="B23" s="9"/>
       <c r="C23" s="9"/>
@@ -1103,7 +1099,7 @@
       <c r="H23" s="16"/>
       <c r="I23" s="16"/>
     </row>
-    <row r="24" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="12"/>
       <c r="B24" s="9"/>
       <c r="C24" s="9"/>
@@ -1114,29 +1110,29 @@
       <c r="H24" s="16"/>
       <c r="I24" s="16"/>
     </row>
-    <row r="25" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="12"/>
       <c r="B25" s="9"/>
       <c r="C25" s="9"/>
       <c r="D25" s="16"/>
-      <c r="E25" s="21"/>
-      <c r="F25" s="21"/>
-      <c r="G25" s="21"/>
-      <c r="H25" s="21"/>
+      <c r="E25" s="16"/>
+      <c r="F25" s="16"/>
+      <c r="G25" s="16"/>
+      <c r="H25" s="16"/>
       <c r="I25" s="16"/>
     </row>
-    <row r="26" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="12"/>
       <c r="B26" s="9"/>
       <c r="C26" s="9"/>
       <c r="D26" s="16"/>
-      <c r="E26" s="21"/>
-      <c r="F26" s="21"/>
-      <c r="G26" s="21"/>
-      <c r="H26" s="21"/>
+      <c r="E26" s="16"/>
+      <c r="F26" s="16"/>
+      <c r="G26" s="16"/>
+      <c r="H26" s="16"/>
       <c r="I26" s="16"/>
     </row>
-    <row r="27" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="16"/>
       <c r="B27" s="9"/>
       <c r="C27" s="9"/>
@@ -1147,7 +1143,7 @@
       <c r="H27" s="16"/>
       <c r="I27" s="16"/>
     </row>
-    <row r="28" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="16"/>
       <c r="B28" s="9"/>
       <c r="C28" s="9"/>
@@ -1158,7 +1154,7 @@
       <c r="H28" s="16"/>
       <c r="I28" s="16"/>
     </row>
-    <row r="29" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="16"/>
       <c r="B29" s="9"/>
       <c r="C29" s="9"/>
@@ -1169,7 +1165,7 @@
       <c r="H29" s="16"/>
       <c r="I29" s="16"/>
     </row>
-    <row r="30" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="16"/>
       <c r="B30" s="9"/>
       <c r="C30" s="9"/>
@@ -1180,7 +1176,7 @@
       <c r="H30" s="16"/>
       <c r="I30" s="16"/>
     </row>
-    <row r="31" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="16"/>
       <c r="B31" s="9"/>
       <c r="C31" s="9"/>
@@ -1191,7 +1187,7 @@
       <c r="H31" s="16"/>
       <c r="I31" s="16"/>
     </row>
-    <row r="32" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="16"/>
       <c r="B32" s="9"/>
       <c r="C32" s="9"/>
@@ -1202,7 +1198,7 @@
       <c r="H32" s="16"/>
       <c r="I32" s="16"/>
     </row>
-    <row r="33" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="16"/>
       <c r="B33" s="9"/>
       <c r="C33" s="9"/>
@@ -1213,7 +1209,7 @@
       <c r="H33" s="16"/>
       <c r="I33" s="16"/>
     </row>
-    <row r="34" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="16"/>
       <c r="B34" s="9"/>
       <c r="C34" s="9"/>
@@ -1224,7 +1220,7 @@
       <c r="H34" s="16"/>
       <c r="I34" s="16"/>
     </row>
-    <row r="35" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="16"/>
       <c r="B35" s="9"/>
       <c r="C35" s="9"/>
@@ -1235,7 +1231,7 @@
       <c r="H35" s="16"/>
       <c r="I35" s="16"/>
     </row>
-    <row r="36" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="14"/>
       <c r="B36" s="20"/>
       <c r="C36" s="20"/>
@@ -1246,7 +1242,7 @@
       <c r="H36" s="14"/>
       <c r="I36" s="14"/>
     </row>
-    <row r="37" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="14"/>
       <c r="B37" s="20"/>
       <c r="C37" s="20"/>
@@ -1257,7 +1253,7 @@
       <c r="H37" s="14"/>
       <c r="I37" s="14"/>
     </row>
-    <row r="38" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="14"/>
       <c r="B38" s="20"/>
       <c r="C38" s="20"/>
@@ -1268,7 +1264,7 @@
       <c r="H38" s="14"/>
       <c r="I38" s="14"/>
     </row>
-    <row r="39" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="14"/>
       <c r="B39" s="20"/>
       <c r="C39" s="20"/>
@@ -1279,7 +1275,7 @@
       <c r="H39" s="14"/>
       <c r="I39" s="14"/>
     </row>
-    <row r="40" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="14"/>
       <c r="B40" s="20"/>
       <c r="C40" s="20"/>
@@ -1290,7 +1286,7 @@
       <c r="H40" s="14"/>
       <c r="I40" s="14"/>
     </row>
-    <row r="41" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="14"/>
       <c r="B41" s="20"/>
       <c r="C41" s="20"/>
@@ -1301,7 +1297,7 @@
       <c r="H41" s="14"/>
       <c r="I41" s="14"/>
     </row>
-    <row r="42" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="14"/>
       <c r="B42" s="20"/>
       <c r="C42" s="20"/>
@@ -1312,7 +1308,7 @@
       <c r="H42" s="14"/>
       <c r="I42" s="14"/>
     </row>
-    <row r="43" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="14"/>
       <c r="B43" s="20"/>
       <c r="C43" s="20"/>
@@ -1323,7 +1319,7 @@
       <c r="H43" s="14"/>
       <c r="I43" s="14"/>
     </row>
-    <row r="44" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="14"/>
       <c r="B44" s="20"/>
       <c r="C44" s="20"/>
@@ -1334,7 +1330,7 @@
       <c r="H44" s="14"/>
       <c r="I44" s="14"/>
     </row>
-    <row r="45" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="14"/>
       <c r="B45" s="20"/>
       <c r="C45" s="20"/>
@@ -1345,7 +1341,7 @@
       <c r="H45" s="14"/>
       <c r="I45" s="14"/>
     </row>
-    <row r="46" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="14"/>
       <c r="B46" s="20"/>
       <c r="C46" s="20"/>
@@ -1356,7 +1352,7 @@
       <c r="H46" s="14"/>
       <c r="I46" s="14"/>
     </row>
-    <row r="47" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="14"/>
       <c r="B47" s="20"/>
       <c r="C47" s="20"/>
@@ -1367,7 +1363,7 @@
       <c r="H47" s="14"/>
       <c r="I47" s="14"/>
     </row>
-    <row r="48" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="14"/>
       <c r="B48" s="20"/>
       <c r="C48" s="20"/>
@@ -1378,7 +1374,7 @@
       <c r="H48" s="14"/>
       <c r="I48" s="14"/>
     </row>
-    <row r="49" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="14"/>
       <c r="B49" s="20"/>
       <c r="C49" s="20"/>
@@ -1389,7 +1385,7 @@
       <c r="H49" s="14"/>
       <c r="I49" s="14"/>
     </row>
-    <row r="50" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="14"/>
       <c r="B50" s="20"/>
       <c r="C50" s="20"/>
@@ -1400,7 +1396,7 @@
       <c r="H50" s="14"/>
       <c r="I50" s="14"/>
     </row>
-    <row r="51" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="14"/>
       <c r="B51" s="20"/>
       <c r="C51" s="20"/>
@@ -1411,7 +1407,7 @@
       <c r="H51" s="14"/>
       <c r="I51" s="14"/>
     </row>
-    <row r="52" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="14"/>
       <c r="B52" s="20"/>
       <c r="C52" s="20"/>
@@ -1422,7 +1418,7 @@
       <c r="H52" s="14"/>
       <c r="I52" s="14"/>
     </row>
-    <row r="53" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="14"/>
       <c r="B53" s="20"/>
       <c r="C53" s="20"/>
@@ -1433,7 +1429,7 @@
       <c r="H53" s="14"/>
       <c r="I53" s="14"/>
     </row>
-    <row r="54" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="14"/>
       <c r="B54" s="20"/>
       <c r="C54" s="20"/>
@@ -1444,7 +1440,7 @@
       <c r="H54" s="14"/>
       <c r="I54" s="14"/>
     </row>
-    <row r="55" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="14"/>
       <c r="B55" s="20"/>
       <c r="C55" s="20"/>
@@ -1455,7 +1451,7 @@
       <c r="H55" s="14"/>
       <c r="I55" s="14"/>
     </row>
-    <row r="56" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="14"/>
       <c r="B56" s="20"/>
       <c r="C56" s="20"/>
@@ -1466,7 +1462,7 @@
       <c r="H56" s="14"/>
       <c r="I56" s="14"/>
     </row>
-    <row r="57" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="14"/>
       <c r="B57" s="20"/>
       <c r="C57" s="20"/>
@@ -1477,7 +1473,7 @@
       <c r="H57" s="14"/>
       <c r="I57" s="14"/>
     </row>
-    <row r="58" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="14"/>
       <c r="B58" s="20"/>
       <c r="C58" s="20"/>
@@ -1488,7 +1484,7 @@
       <c r="H58" s="14"/>
       <c r="I58" s="14"/>
     </row>
-    <row r="59" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="14"/>
       <c r="B59" s="20"/>
       <c r="C59" s="20"/>
@@ -1499,7 +1495,7 @@
       <c r="H59" s="14"/>
       <c r="I59" s="14"/>
     </row>
-    <row r="60" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="14"/>
       <c r="B60" s="20"/>
       <c r="C60" s="20"/>
@@ -1510,7 +1506,7 @@
       <c r="H60" s="14"/>
       <c r="I60" s="14"/>
     </row>
-    <row r="61" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="14"/>
       <c r="B61" s="20"/>
       <c r="C61" s="20"/>
@@ -1521,7 +1517,7 @@
       <c r="H61" s="14"/>
       <c r="I61" s="14"/>
     </row>
-    <row r="62" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="14"/>
       <c r="B62" s="20"/>
       <c r="C62" s="20"/>
@@ -1532,7 +1528,7 @@
       <c r="H62" s="14"/>
       <c r="I62" s="14"/>
     </row>
-    <row r="63" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="14"/>
       <c r="B63" s="20"/>
       <c r="C63" s="20"/>
@@ -1543,7 +1539,7 @@
       <c r="H63" s="14"/>
       <c r="I63" s="14"/>
     </row>
-    <row r="64" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="14"/>
       <c r="B64" s="20"/>
       <c r="C64" s="20"/>
@@ -1554,7 +1550,7 @@
       <c r="H64" s="14"/>
       <c r="I64" s="14"/>
     </row>
-    <row r="65" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="14"/>
       <c r="B65" s="20"/>
       <c r="C65" s="20"/>
@@ -1565,7 +1561,7 @@
       <c r="H65" s="14"/>
       <c r="I65" s="14"/>
     </row>
-    <row r="66" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="14"/>
       <c r="B66" s="20"/>
       <c r="C66" s="20"/>
@@ -1576,7 +1572,7 @@
       <c r="H66" s="14"/>
       <c r="I66" s="14"/>
     </row>
-    <row r="67" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="14"/>
       <c r="B67" s="20"/>
       <c r="C67" s="20"/>
@@ -1587,7 +1583,7 @@
       <c r="H67" s="14"/>
       <c r="I67" s="14"/>
     </row>
-    <row r="68" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="14"/>
       <c r="B68" s="20"/>
       <c r="C68" s="20"/>
@@ -1598,7 +1594,7 @@
       <c r="H68" s="14"/>
       <c r="I68" s="14"/>
     </row>
-    <row r="69" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="14"/>
       <c r="B69" s="20"/>
       <c r="C69" s="20"/>
@@ -1609,7 +1605,7 @@
       <c r="H69" s="14"/>
       <c r="I69" s="14"/>
     </row>
-    <row r="70" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="14"/>
       <c r="B70" s="20"/>
       <c r="C70" s="20"/>
@@ -1620,7 +1616,7 @@
       <c r="H70" s="14"/>
       <c r="I70" s="14"/>
     </row>
-    <row r="71" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="14"/>
       <c r="B71" s="20"/>
       <c r="C71" s="20"/>
@@ -1631,7 +1627,7 @@
       <c r="H71" s="14"/>
       <c r="I71" s="14"/>
     </row>
-    <row r="72" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="14"/>
       <c r="B72" s="20"/>
       <c r="C72" s="20"/>
@@ -1642,7 +1638,7 @@
       <c r="H72" s="14"/>
       <c r="I72" s="14"/>
     </row>
-    <row r="73" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="14"/>
       <c r="B73" s="20"/>
       <c r="C73" s="20"/>
@@ -1653,7 +1649,7 @@
       <c r="H73" s="14"/>
       <c r="I73" s="14"/>
     </row>
-    <row r="74" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="14"/>
       <c r="B74" s="20"/>
       <c r="C74" s="20"/>
@@ -1664,7 +1660,7 @@
       <c r="H74" s="14"/>
       <c r="I74" s="14"/>
     </row>
-    <row r="75" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="14"/>
       <c r="B75" s="20"/>
       <c r="C75" s="20"/>
@@ -1675,7 +1671,7 @@
       <c r="H75" s="14"/>
       <c r="I75" s="14"/>
     </row>
-    <row r="76" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="14"/>
       <c r="B76" s="20"/>
       <c r="C76" s="20"/>
@@ -1686,7 +1682,7 @@
       <c r="H76" s="14"/>
       <c r="I76" s="14"/>
     </row>
-    <row r="77" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="14"/>
       <c r="B77" s="20"/>
       <c r="C77" s="20"/>
@@ -1697,7 +1693,7 @@
       <c r="H77" s="14"/>
       <c r="I77" s="14"/>
     </row>
-    <row r="78" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="14"/>
       <c r="B78" s="20"/>
       <c r="C78" s="20"/>
@@ -1708,7 +1704,7 @@
       <c r="H78" s="14"/>
       <c r="I78" s="14"/>
     </row>
-    <row r="79" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="14"/>
       <c r="B79" s="20"/>
       <c r="C79" s="20"/>
@@ -1719,7 +1715,7 @@
       <c r="H79" s="14"/>
       <c r="I79" s="14"/>
     </row>
-    <row r="80" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="14"/>
       <c r="B80" s="20"/>
       <c r="C80" s="20"/>
@@ -1730,7 +1726,7 @@
       <c r="H80" s="14"/>
       <c r="I80" s="14"/>
     </row>
-    <row r="81" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="14"/>
       <c r="B81" s="20"/>
       <c r="C81" s="20"/>
@@ -1741,7 +1737,7 @@
       <c r="H81" s="14"/>
       <c r="I81" s="14"/>
     </row>
-    <row r="82" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="14"/>
       <c r="B82" s="20"/>
       <c r="C82" s="20"/>
@@ -1752,7 +1748,7 @@
       <c r="H82" s="14"/>
       <c r="I82" s="14"/>
     </row>
-    <row r="83" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="14"/>
       <c r="B83" s="20"/>
       <c r="C83" s="20"/>
@@ -1763,7 +1759,7 @@
       <c r="H83" s="14"/>
       <c r="I83" s="14"/>
     </row>
-    <row r="84" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="14"/>
       <c r="B84" s="20"/>
       <c r="C84" s="20"/>
@@ -1774,7 +1770,7 @@
       <c r="H84" s="14"/>
       <c r="I84" s="14"/>
     </row>
-    <row r="85" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="14"/>
       <c r="B85" s="20"/>
       <c r="C85" s="20"/>
@@ -1785,7 +1781,7 @@
       <c r="H85" s="14"/>
       <c r="I85" s="14"/>
     </row>
-    <row r="86" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="14"/>
       <c r="B86" s="20"/>
       <c r="C86" s="20"/>
@@ -1796,7 +1792,7 @@
       <c r="H86" s="14"/>
       <c r="I86" s="14"/>
     </row>
-    <row r="87" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="14"/>
       <c r="B87" s="20"/>
       <c r="C87" s="20"/>
@@ -1807,7 +1803,7 @@
       <c r="H87" s="14"/>
       <c r="I87" s="14"/>
     </row>
-    <row r="88" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="14"/>
       <c r="B88" s="20"/>
       <c r="C88" s="20"/>
@@ -1818,7 +1814,7 @@
       <c r="H88" s="14"/>
       <c r="I88" s="14"/>
     </row>
-    <row r="89" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="14"/>
       <c r="B89" s="20"/>
       <c r="C89" s="20"/>
@@ -1829,7 +1825,7 @@
       <c r="H89" s="14"/>
       <c r="I89" s="14"/>
     </row>
-    <row r="90" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="14"/>
       <c r="B90" s="20"/>
       <c r="C90" s="20"/>
@@ -1840,7 +1836,7 @@
       <c r="H90" s="14"/>
       <c r="I90" s="14"/>
     </row>
-    <row r="91" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="14"/>
       <c r="B91" s="20"/>
       <c r="C91" s="20"/>
@@ -1851,7 +1847,7 @@
       <c r="H91" s="14"/>
       <c r="I91" s="14"/>
     </row>
-    <row r="92" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="14"/>
       <c r="B92" s="20"/>
       <c r="C92" s="20"/>
@@ -1862,7 +1858,7 @@
       <c r="H92" s="14"/>
       <c r="I92" s="14"/>
     </row>
-    <row r="93" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="14"/>
       <c r="B93" s="20"/>
       <c r="C93" s="20"/>
@@ -1873,7 +1869,7 @@
       <c r="H93" s="14"/>
       <c r="I93" s="14"/>
     </row>
-    <row r="94" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="14"/>
       <c r="B94" s="20"/>
       <c r="C94" s="20"/>
@@ -1884,7 +1880,7 @@
       <c r="H94" s="14"/>
       <c r="I94" s="14"/>
     </row>
-    <row r="95" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="14"/>
       <c r="B95" s="20"/>
       <c r="C95" s="20"/>
@@ -1895,7 +1891,7 @@
       <c r="H95" s="14"/>
       <c r="I95" s="14"/>
     </row>
-    <row r="96" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="14"/>
       <c r="B96" s="20"/>
       <c r="C96" s="20"/>
@@ -1906,7 +1902,7 @@
       <c r="H96" s="14"/>
       <c r="I96" s="14"/>
     </row>
-    <row r="97" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="14"/>
       <c r="B97" s="20"/>
       <c r="C97" s="20"/>
@@ -1917,7 +1913,7 @@
       <c r="H97" s="14"/>
       <c r="I97" s="14"/>
     </row>
-    <row r="98" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="14"/>
       <c r="B98" s="20"/>
       <c r="C98" s="20"/>
@@ -1928,7 +1924,7 @@
       <c r="H98" s="14"/>
       <c r="I98" s="14"/>
     </row>
-    <row r="99" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="14"/>
       <c r="B99" s="20"/>
       <c r="C99" s="20"/>
@@ -1939,7 +1935,7 @@
       <c r="H99" s="14"/>
       <c r="I99" s="14"/>
     </row>
-    <row r="100" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="14"/>
       <c r="B100" s="20"/>
       <c r="C100" s="20"/>
@@ -1950,7 +1946,7 @@
       <c r="H100" s="14"/>
       <c r="I100" s="14"/>
     </row>
-    <row r="101" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="14"/>
       <c r="B101" s="20"/>
       <c r="C101" s="20"/>
@@ -1961,7 +1957,7 @@
       <c r="H101" s="14"/>
       <c r="I101" s="14"/>
     </row>
-    <row r="102" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A102" s="14"/>
       <c r="B102" s="20"/>
       <c r="C102" s="20"/>
@@ -1972,7 +1968,7 @@
       <c r="H102" s="14"/>
       <c r="I102" s="14"/>
     </row>
-    <row r="103" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="14"/>
       <c r="B103" s="20"/>
       <c r="C103" s="20"/>
@@ -1983,7 +1979,7 @@
       <c r="H103" s="14"/>
       <c r="I103" s="14"/>
     </row>
-    <row r="104" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="14"/>
       <c r="B104" s="20"/>
       <c r="C104" s="20"/>
@@ -1994,7 +1990,7 @@
       <c r="H104" s="14"/>
       <c r="I104" s="14"/>
     </row>
-    <row r="105" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="14"/>
       <c r="B105" s="20"/>
       <c r="C105" s="20"/>
@@ -2005,7 +2001,7 @@
       <c r="H105" s="14"/>
       <c r="I105" s="14"/>
     </row>
-    <row r="106" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A106" s="14"/>
       <c r="B106" s="20"/>
       <c r="C106" s="20"/>
@@ -2016,7 +2012,7 @@
       <c r="H106" s="14"/>
       <c r="I106" s="14"/>
     </row>
-    <row r="107" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" s="14"/>
       <c r="B107" s="20"/>
       <c r="C107" s="20"/>
@@ -2027,7 +2023,7 @@
       <c r="H107" s="14"/>
       <c r="I107" s="14"/>
     </row>
-    <row r="108" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108" s="14"/>
       <c r="B108" s="20"/>
       <c r="C108" s="20"/>
@@ -2038,7 +2034,7 @@
       <c r="H108" s="14"/>
       <c r="I108" s="14"/>
     </row>
-    <row r="109" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A109" s="14"/>
       <c r="B109" s="20"/>
       <c r="C109" s="20"/>
@@ -2049,7 +2045,7 @@
       <c r="H109" s="14"/>
       <c r="I109" s="14"/>
     </row>
-    <row r="110" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110" s="14"/>
       <c r="B110" s="20"/>
       <c r="C110" s="20"/>
@@ -2060,7 +2056,7 @@
       <c r="H110" s="14"/>
       <c r="I110" s="14"/>
     </row>
-    <row r="111" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A111" s="14"/>
       <c r="B111" s="20"/>
       <c r="C111" s="20"/>
@@ -2071,7 +2067,7 @@
       <c r="H111" s="14"/>
       <c r="I111" s="14"/>
     </row>
-    <row r="112" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A112" s="14"/>
       <c r="B112" s="20"/>
       <c r="C112" s="20"/>
@@ -2082,7 +2078,7 @@
       <c r="H112" s="14"/>
       <c r="I112" s="14"/>
     </row>
-    <row r="113" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A113" s="14"/>
       <c r="B113" s="20"/>
       <c r="C113" s="20"/>
@@ -2093,7 +2089,7 @@
       <c r="H113" s="14"/>
       <c r="I113" s="14"/>
     </row>
-    <row r="114" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A114" s="14"/>
       <c r="B114" s="20"/>
       <c r="C114" s="20"/>
@@ -2104,7 +2100,7 @@
       <c r="H114" s="14"/>
       <c r="I114" s="14"/>
     </row>
-    <row r="115" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A115" s="14"/>
       <c r="B115" s="20"/>
       <c r="C115" s="20"/>
@@ -2115,7 +2111,7 @@
       <c r="H115" s="14"/>
       <c r="I115" s="14"/>
     </row>
-    <row r="116" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116" s="14"/>
       <c r="B116" s="20"/>
       <c r="C116" s="20"/>
@@ -2126,7 +2122,7 @@
       <c r="H116" s="14"/>
       <c r="I116" s="14"/>
     </row>
-    <row r="117" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="14"/>
       <c r="B117" s="20"/>
       <c r="C117" s="20"/>
@@ -2137,7 +2133,7 @@
       <c r="H117" s="14"/>
       <c r="I117" s="14"/>
     </row>
-    <row r="118" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A118" s="14"/>
       <c r="B118" s="20"/>
       <c r="C118" s="20"/>
@@ -2148,7 +2144,7 @@
       <c r="H118" s="14"/>
       <c r="I118" s="14"/>
     </row>
-    <row r="119" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A119" s="14"/>
       <c r="B119" s="20"/>
       <c r="C119" s="20"/>
@@ -2159,7 +2155,7 @@
       <c r="H119" s="14"/>
       <c r="I119" s="14"/>
     </row>
-    <row r="120" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="14"/>
       <c r="B120" s="20"/>
       <c r="C120" s="20"/>
@@ -2170,7 +2166,7 @@
       <c r="H120" s="14"/>
       <c r="I120" s="14"/>
     </row>
-    <row r="121" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A121" s="14"/>
       <c r="B121" s="20"/>
       <c r="C121" s="20"/>
@@ -2181,7 +2177,7 @@
       <c r="H121" s="14"/>
       <c r="I121" s="14"/>
     </row>
-    <row r="122" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A122" s="14"/>
       <c r="B122" s="20"/>
       <c r="C122" s="20"/>
@@ -2192,7 +2188,7 @@
       <c r="H122" s="14"/>
       <c r="I122" s="14"/>
     </row>
-    <row r="123" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A123" s="14"/>
       <c r="B123" s="20"/>
       <c r="C123" s="20"/>
@@ -2203,7 +2199,7 @@
       <c r="H123" s="14"/>
       <c r="I123" s="14"/>
     </row>
-    <row r="124" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A124" s="14"/>
       <c r="B124" s="20"/>
       <c r="C124" s="20"/>
@@ -2214,7 +2210,7 @@
       <c r="H124" s="14"/>
       <c r="I124" s="14"/>
     </row>
-    <row r="125" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A125" s="14"/>
       <c r="B125" s="20"/>
       <c r="C125" s="20"/>
@@ -2225,7 +2221,7 @@
       <c r="H125" s="14"/>
       <c r="I125" s="14"/>
     </row>
-    <row r="126" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A126" s="14"/>
       <c r="B126" s="20"/>
       <c r="C126" s="20"/>
@@ -2236,7 +2232,7 @@
       <c r="H126" s="14"/>
       <c r="I126" s="14"/>
     </row>
-    <row r="127" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A127" s="14"/>
       <c r="B127" s="20"/>
       <c r="C127" s="20"/>
@@ -2247,7 +2243,7 @@
       <c r="H127" s="14"/>
       <c r="I127" s="14"/>
     </row>
-    <row r="128" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A128" s="14"/>
       <c r="B128" s="20"/>
       <c r="C128" s="20"/>
@@ -2258,7 +2254,7 @@
       <c r="H128" s="14"/>
       <c r="I128" s="14"/>
     </row>
-    <row r="129" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A129" s="14"/>
       <c r="B129" s="20"/>
       <c r="C129" s="20"/>
@@ -2269,7 +2265,7 @@
       <c r="H129" s="14"/>
       <c r="I129" s="14"/>
     </row>
-    <row r="130" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A130" s="14"/>
       <c r="B130" s="20"/>
       <c r="C130" s="20"/>
@@ -2280,7 +2276,7 @@
       <c r="H130" s="14"/>
       <c r="I130" s="14"/>
     </row>
-    <row r="131" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A131" s="14"/>
       <c r="B131" s="20"/>
       <c r="C131" s="20"/>
@@ -2291,7 +2287,7 @@
       <c r="H131" s="14"/>
       <c r="I131" s="14"/>
     </row>
-    <row r="132" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A132" s="14"/>
       <c r="B132" s="20"/>
       <c r="C132" s="20"/>
@@ -2302,7 +2298,7 @@
       <c r="H132" s="14"/>
       <c r="I132" s="14"/>
     </row>
-    <row r="133" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A133" s="14"/>
       <c r="B133" s="20"/>
       <c r="C133" s="20"/>
@@ -2313,7 +2309,7 @@
       <c r="H133" s="14"/>
       <c r="I133" s="14"/>
     </row>
-    <row r="134" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A134" s="14"/>
       <c r="B134" s="20"/>
       <c r="C134" s="20"/>
@@ -2324,7 +2320,7 @@
       <c r="H134" s="14"/>
       <c r="I134" s="14"/>
     </row>
-    <row r="135" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A135" s="14"/>
       <c r="B135" s="20"/>
       <c r="C135" s="20"/>
@@ -2335,7 +2331,7 @@
       <c r="H135" s="14"/>
       <c r="I135" s="14"/>
     </row>
-    <row r="136" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A136" s="14"/>
       <c r="B136" s="20"/>
       <c r="C136" s="20"/>
@@ -2346,7 +2342,7 @@
       <c r="H136" s="14"/>
       <c r="I136" s="14"/>
     </row>
-    <row r="137" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A137" s="14"/>
       <c r="B137" s="20"/>
       <c r="C137" s="20"/>
@@ -2357,7 +2353,7 @@
       <c r="H137" s="14"/>
       <c r="I137" s="14"/>
     </row>
-    <row r="138" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A138" s="14"/>
       <c r="B138" s="20"/>
       <c r="C138" s="20"/>
@@ -2368,7 +2364,7 @@
       <c r="H138" s="14"/>
       <c r="I138" s="14"/>
     </row>
-    <row r="139" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A139" s="14"/>
       <c r="B139" s="20"/>
       <c r="C139" s="20"/>
@@ -2379,7 +2375,7 @@
       <c r="H139" s="14"/>
       <c r="I139" s="14"/>
     </row>
-    <row r="140" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A140" s="14"/>
       <c r="B140" s="20"/>
       <c r="C140" s="20"/>
@@ -2390,7 +2386,7 @@
       <c r="H140" s="14"/>
       <c r="I140" s="14"/>
     </row>
-    <row r="141" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A141" s="14"/>
       <c r="B141" s="20"/>
       <c r="C141" s="20"/>
@@ -2401,7 +2397,7 @@
       <c r="H141" s="14"/>
       <c r="I141" s="14"/>
     </row>
-    <row r="142" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A142" s="14"/>
       <c r="B142" s="20"/>
       <c r="C142" s="20"/>
@@ -2412,7 +2408,7 @@
       <c r="H142" s="14"/>
       <c r="I142" s="14"/>
     </row>
-    <row r="143" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A143" s="14"/>
       <c r="B143" s="20"/>
       <c r="C143" s="20"/>
@@ -2423,7 +2419,7 @@
       <c r="H143" s="14"/>
       <c r="I143" s="14"/>
     </row>
-    <row r="144" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A144" s="14"/>
       <c r="B144" s="20"/>
       <c r="C144" s="20"/>
@@ -2434,7 +2430,7 @@
       <c r="H144" s="14"/>
       <c r="I144" s="14"/>
     </row>
-    <row r="145" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A145" s="14"/>
       <c r="B145" s="20"/>
       <c r="C145" s="20"/>
@@ -2445,7 +2441,7 @@
       <c r="H145" s="14"/>
       <c r="I145" s="14"/>
     </row>
-    <row r="146" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A146" s="14"/>
       <c r="B146" s="20"/>
       <c r="C146" s="20"/>
@@ -2456,7 +2452,7 @@
       <c r="H146" s="14"/>
       <c r="I146" s="14"/>
     </row>
-    <row r="147" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A147" s="14"/>
       <c r="B147" s="20"/>
       <c r="C147" s="20"/>
@@ -2467,7 +2463,7 @@
       <c r="H147" s="14"/>
       <c r="I147" s="14"/>
     </row>
-    <row r="148" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A148" s="14"/>
       <c r="B148" s="20"/>
       <c r="C148" s="20"/>
@@ -2478,7 +2474,7 @@
       <c r="H148" s="14"/>
       <c r="I148" s="14"/>
     </row>
-    <row r="149" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A149" s="14"/>
       <c r="B149" s="20"/>
       <c r="C149" s="20"/>
@@ -2489,7 +2485,7 @@
       <c r="H149" s="14"/>
       <c r="I149" s="14"/>
     </row>
-    <row r="150" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A150" s="14"/>
       <c r="B150" s="20"/>
       <c r="C150" s="20"/>
@@ -2500,7 +2496,7 @@
       <c r="H150" s="14"/>
       <c r="I150" s="14"/>
     </row>
-    <row r="151" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A151" s="14"/>
       <c r="B151" s="20"/>
       <c r="C151" s="20"/>
@@ -2511,7 +2507,7 @@
       <c r="H151" s="14"/>
       <c r="I151" s="14"/>
     </row>
-    <row r="152" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A152" s="14"/>
       <c r="B152" s="20"/>
       <c r="C152" s="20"/>
@@ -2522,7 +2518,7 @@
       <c r="H152" s="14"/>
       <c r="I152" s="14"/>
     </row>
-    <row r="153" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A153" s="14"/>
       <c r="B153" s="20"/>
       <c r="C153" s="20"/>
@@ -2533,7 +2529,7 @@
       <c r="H153" s="14"/>
       <c r="I153" s="14"/>
     </row>
-    <row r="154" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A154" s="14"/>
       <c r="B154" s="20"/>
       <c r="C154" s="20"/>
@@ -2544,7 +2540,7 @@
       <c r="H154" s="14"/>
       <c r="I154" s="14"/>
     </row>
-    <row r="155" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A155" s="14"/>
       <c r="B155" s="20"/>
       <c r="C155" s="20"/>
@@ -2555,7 +2551,7 @@
       <c r="H155" s="14"/>
       <c r="I155" s="14"/>
     </row>
-    <row r="156" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A156" s="14"/>
       <c r="B156" s="20"/>
       <c r="C156" s="20"/>
@@ -2566,7 +2562,7 @@
       <c r="H156" s="14"/>
       <c r="I156" s="14"/>
     </row>
-    <row r="157" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A157" s="14"/>
       <c r="B157" s="20"/>
       <c r="C157" s="20"/>
@@ -2577,7 +2573,7 @@
       <c r="H157" s="14"/>
       <c r="I157" s="14"/>
     </row>
-    <row r="158" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A158" s="14"/>
       <c r="B158" s="20"/>
       <c r="C158" s="20"/>
@@ -2588,7 +2584,7 @@
       <c r="H158" s="14"/>
       <c r="I158" s="14"/>
     </row>
-    <row r="159" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A159" s="14"/>
       <c r="B159" s="20"/>
       <c r="C159" s="20"/>
@@ -2599,7 +2595,7 @@
       <c r="H159" s="14"/>
       <c r="I159" s="14"/>
     </row>
-    <row r="160" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A160" s="14"/>
       <c r="B160" s="20"/>
       <c r="C160" s="20"/>
@@ -2610,7 +2606,7 @@
       <c r="H160" s="14"/>
       <c r="I160" s="14"/>
     </row>
-    <row r="161" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A161" s="14"/>
       <c r="B161" s="20"/>
       <c r="C161" s="20"/>
@@ -2621,7 +2617,7 @@
       <c r="H161" s="14"/>
       <c r="I161" s="14"/>
     </row>
-    <row r="162" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A162" s="14"/>
       <c r="B162" s="20"/>
       <c r="C162" s="20"/>
@@ -2632,7 +2628,7 @@
       <c r="H162" s="14"/>
       <c r="I162" s="14"/>
     </row>
-    <row r="163" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A163" s="14"/>
       <c r="B163" s="20"/>
       <c r="C163" s="20"/>
@@ -2643,7 +2639,7 @@
       <c r="H163" s="14"/>
       <c r="I163" s="14"/>
     </row>
-    <row r="164" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A164" s="14"/>
       <c r="B164" s="20"/>
       <c r="C164" s="20"/>
@@ -2654,7 +2650,7 @@
       <c r="H164" s="14"/>
       <c r="I164" s="14"/>
     </row>
-    <row r="165" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A165" s="14"/>
       <c r="B165" s="20"/>
       <c r="C165" s="20"/>
@@ -2665,7 +2661,7 @@
       <c r="H165" s="14"/>
       <c r="I165" s="14"/>
     </row>
-    <row r="166" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A166" s="14"/>
       <c r="B166" s="20"/>
       <c r="C166" s="20"/>
@@ -2676,7 +2672,7 @@
       <c r="H166" s="14"/>
       <c r="I166" s="14"/>
     </row>
-    <row r="167" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A167" s="14"/>
       <c r="B167" s="20"/>
       <c r="C167" s="20"/>
@@ -2687,7 +2683,7 @@
       <c r="H167" s="14"/>
       <c r="I167" s="14"/>
     </row>
-    <row r="168" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A168" s="14"/>
       <c r="B168" s="20"/>
       <c r="C168" s="20"/>
@@ -2698,7 +2694,7 @@
       <c r="H168" s="14"/>
       <c r="I168" s="14"/>
     </row>
-    <row r="169" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A169" s="14"/>
       <c r="B169" s="20"/>
       <c r="C169" s="20"/>
@@ -2709,7 +2705,7 @@
       <c r="H169" s="14"/>
       <c r="I169" s="14"/>
     </row>
-    <row r="170" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A170" s="14"/>
       <c r="B170" s="20"/>
       <c r="C170" s="20"/>
@@ -2720,7 +2716,7 @@
       <c r="H170" s="14"/>
       <c r="I170" s="14"/>
     </row>
-    <row r="171" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A171" s="14"/>
       <c r="B171" s="20"/>
       <c r="C171" s="20"/>
@@ -2731,7 +2727,7 @@
       <c r="H171" s="14"/>
       <c r="I171" s="14"/>
     </row>
-    <row r="172" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A172" s="14"/>
       <c r="B172" s="20"/>
       <c r="C172" s="20"/>
@@ -2742,7 +2738,7 @@
       <c r="H172" s="14"/>
       <c r="I172" s="14"/>
     </row>
-    <row r="173" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A173" s="14"/>
       <c r="B173" s="20"/>
       <c r="C173" s="20"/>
@@ -2753,7 +2749,7 @@
       <c r="H173" s="14"/>
       <c r="I173" s="14"/>
     </row>
-    <row r="174" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A174" s="14"/>
       <c r="B174" s="20"/>
       <c r="C174" s="20"/>
@@ -2764,7 +2760,7 @@
       <c r="H174" s="14"/>
       <c r="I174" s="14"/>
     </row>
-    <row r="175" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A175" s="14"/>
       <c r="B175" s="20"/>
       <c r="C175" s="20"/>
@@ -2775,7 +2771,7 @@
       <c r="H175" s="14"/>
       <c r="I175" s="14"/>
     </row>
-    <row r="176" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A176" s="14"/>
       <c r="B176" s="20"/>
       <c r="C176" s="20"/>
@@ -2786,7 +2782,7 @@
       <c r="H176" s="14"/>
       <c r="I176" s="14"/>
     </row>
-    <row r="177" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A177" s="14"/>
       <c r="B177" s="20"/>
       <c r="C177" s="20"/>
@@ -2797,7 +2793,7 @@
       <c r="H177" s="14"/>
       <c r="I177" s="14"/>
     </row>
-    <row r="178" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A178" s="14"/>
       <c r="B178" s="20"/>
       <c r="C178" s="20"/>
@@ -2808,7 +2804,7 @@
       <c r="H178" s="14"/>
       <c r="I178" s="14"/>
     </row>
-    <row r="179" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A179" s="14"/>
       <c r="B179" s="20"/>
       <c r="C179" s="20"/>
@@ -2819,7 +2815,7 @@
       <c r="H179" s="14"/>
       <c r="I179" s="14"/>
     </row>
-    <row r="180" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A180" s="14"/>
       <c r="B180" s="20"/>
       <c r="C180" s="20"/>
@@ -2830,7 +2826,7 @@
       <c r="H180" s="14"/>
       <c r="I180" s="14"/>
     </row>
-    <row r="181" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A181" s="14"/>
       <c r="B181" s="20"/>
       <c r="C181" s="20"/>
@@ -2841,7 +2837,7 @@
       <c r="H181" s="14"/>
       <c r="I181" s="14"/>
     </row>
-    <row r="182" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A182" s="14"/>
       <c r="B182" s="20"/>
       <c r="C182" s="20"/>
@@ -2852,7 +2848,7 @@
       <c r="H182" s="14"/>
       <c r="I182" s="14"/>
     </row>
-    <row r="183" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A183" s="14"/>
       <c r="B183" s="20"/>
       <c r="C183" s="20"/>
@@ -2863,7 +2859,7 @@
       <c r="H183" s="14"/>
       <c r="I183" s="14"/>
     </row>
-    <row r="184" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A184" s="14"/>
       <c r="B184" s="20"/>
       <c r="C184" s="20"/>
@@ -2874,7 +2870,7 @@
       <c r="H184" s="14"/>
       <c r="I184" s="14"/>
     </row>
-    <row r="185" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A185" s="14"/>
       <c r="B185" s="20"/>
       <c r="C185" s="20"/>
@@ -2885,7 +2881,7 @@
       <c r="H185" s="14"/>
       <c r="I185" s="14"/>
     </row>
-    <row r="186" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A186" s="14"/>
       <c r="B186" s="20"/>
       <c r="C186" s="20"/>
@@ -2896,7 +2892,7 @@
       <c r="H186" s="14"/>
       <c r="I186" s="14"/>
     </row>
-    <row r="187" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A187" s="14"/>
       <c r="B187" s="20"/>
       <c r="C187" s="20"/>
@@ -2907,7 +2903,7 @@
       <c r="H187" s="14"/>
       <c r="I187" s="14"/>
     </row>
-    <row r="188" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A188" s="14"/>
       <c r="B188" s="20"/>
       <c r="C188" s="20"/>
@@ -2918,7 +2914,7 @@
       <c r="H188" s="14"/>
       <c r="I188" s="14"/>
     </row>
-    <row r="189" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A189" s="14"/>
       <c r="B189" s="20"/>
       <c r="C189" s="20"/>
@@ -2929,7 +2925,7 @@
       <c r="H189" s="14"/>
       <c r="I189" s="14"/>
     </row>
-    <row r="190" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A190" s="14"/>
       <c r="B190" s="20"/>
       <c r="C190" s="20"/>
@@ -2940,7 +2936,7 @@
       <c r="H190" s="14"/>
       <c r="I190" s="14"/>
     </row>
-    <row r="191" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A191" s="14"/>
       <c r="B191" s="20"/>
       <c r="C191" s="20"/>
@@ -2951,7 +2947,7 @@
       <c r="H191" s="14"/>
       <c r="I191" s="14"/>
     </row>
-    <row r="192" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A192" s="14"/>
       <c r="B192" s="20"/>
       <c r="C192" s="20"/>
@@ -2962,7 +2958,7 @@
       <c r="H192" s="14"/>
       <c r="I192" s="14"/>
     </row>
-    <row r="193" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A193" s="14"/>
       <c r="B193" s="20"/>
       <c r="C193" s="20"/>
@@ -2973,7 +2969,7 @@
       <c r="H193" s="14"/>
       <c r="I193" s="14"/>
     </row>
-    <row r="194" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A194" s="14"/>
       <c r="B194" s="20"/>
       <c r="C194" s="20"/>
@@ -2984,7 +2980,7 @@
       <c r="H194" s="14"/>
       <c r="I194" s="14"/>
     </row>
-    <row r="195" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A195" s="14"/>
       <c r="B195" s="20"/>
       <c r="C195" s="20"/>
@@ -2995,7 +2991,7 @@
       <c r="H195" s="14"/>
       <c r="I195" s="14"/>
     </row>
-    <row r="196" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A196" s="14"/>
       <c r="B196" s="20"/>
       <c r="C196" s="20"/>
@@ -3006,7 +3002,7 @@
       <c r="H196" s="14"/>
       <c r="I196" s="14"/>
     </row>
-    <row r="197" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A197" s="14"/>
       <c r="B197" s="20"/>
       <c r="C197" s="20"/>
@@ -3017,7 +3013,7 @@
       <c r="H197" s="14"/>
       <c r="I197" s="14"/>
     </row>
-    <row r="198" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A198" s="14"/>
       <c r="B198" s="20"/>
       <c r="C198" s="20"/>
@@ -3028,7 +3024,7 @@
       <c r="H198" s="14"/>
       <c r="I198" s="14"/>
     </row>
-    <row r="199" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A199" s="14"/>
       <c r="B199" s="20"/>
       <c r="C199" s="20"/>
@@ -3039,7 +3035,7 @@
       <c r="H199" s="14"/>
       <c r="I199" s="14"/>
     </row>
-    <row r="200" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A200" s="14"/>
       <c r="B200" s="20"/>
       <c r="C200" s="20"/>
@@ -3050,7 +3046,7 @@
       <c r="H200" s="14"/>
       <c r="I200" s="14"/>
     </row>
-    <row r="201" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A201" s="14"/>
       <c r="B201" s="20"/>
       <c r="C201" s="20"/>
@@ -3061,7 +3057,7 @@
       <c r="H201" s="14"/>
       <c r="I201" s="14"/>
     </row>
-    <row r="202" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="202" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A202" s="14"/>
       <c r="B202" s="20"/>
       <c r="C202" s="20"/>
@@ -3072,7 +3068,7 @@
       <c r="H202" s="14"/>
       <c r="I202" s="14"/>
     </row>
-    <row r="203" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="203" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A203" s="14"/>
       <c r="B203" s="20"/>
       <c r="C203" s="20"/>
@@ -3083,7 +3079,7 @@
       <c r="H203" s="14"/>
       <c r="I203" s="14"/>
     </row>
-    <row r="204" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A204" s="14"/>
       <c r="B204" s="20"/>
       <c r="C204" s="20"/>
@@ -3094,7 +3090,7 @@
       <c r="H204" s="14"/>
       <c r="I204" s="14"/>
     </row>
-    <row r="205" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="205" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A205" s="14"/>
       <c r="B205" s="20"/>
       <c r="C205" s="20"/>
@@ -3105,7 +3101,7 @@
       <c r="H205" s="14"/>
       <c r="I205" s="14"/>
     </row>
-    <row r="206" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="206" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A206" s="14"/>
       <c r="B206" s="20"/>
       <c r="C206" s="20"/>
@@ -3116,7 +3112,7 @@
       <c r="H206" s="14"/>
       <c r="I206" s="14"/>
     </row>
-    <row r="207" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="207" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A207" s="14"/>
       <c r="B207" s="20"/>
       <c r="C207" s="20"/>
@@ -3127,7 +3123,7 @@
       <c r="H207" s="14"/>
       <c r="I207" s="14"/>
     </row>
-    <row r="208" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="208" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A208" s="14"/>
       <c r="B208" s="20"/>
       <c r="C208" s="20"/>
@@ -3138,7 +3134,7 @@
       <c r="H208" s="14"/>
       <c r="I208" s="14"/>
     </row>
-    <row r="209" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="209" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A209" s="14"/>
       <c r="B209" s="20"/>
       <c r="C209" s="20"/>
@@ -3149,7 +3145,7 @@
       <c r="H209" s="14"/>
       <c r="I209" s="14"/>
     </row>
-    <row r="210" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A210" s="14"/>
       <c r="B210" s="20"/>
       <c r="C210" s="20"/>
@@ -3160,7 +3156,7 @@
       <c r="H210" s="14"/>
       <c r="I210" s="14"/>
     </row>
-    <row r="211" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="211" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A211" s="14"/>
       <c r="B211" s="20"/>
       <c r="C211" s="20"/>
@@ -3171,7 +3167,7 @@
       <c r="H211" s="14"/>
       <c r="I211" s="14"/>
     </row>
-    <row r="212" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="212" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A212" s="14"/>
       <c r="B212" s="20"/>
       <c r="C212" s="20"/>
@@ -3182,7 +3178,7 @@
       <c r="H212" s="14"/>
       <c r="I212" s="14"/>
     </row>
-    <row r="213" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="213" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A213" s="14"/>
       <c r="B213" s="20"/>
       <c r="C213" s="20"/>
@@ -3193,7 +3189,7 @@
       <c r="H213" s="14"/>
       <c r="I213" s="14"/>
     </row>
-    <row r="214" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A214" s="14"/>
       <c r="B214" s="20"/>
       <c r="C214" s="20"/>
@@ -3204,7 +3200,7 @@
       <c r="H214" s="14"/>
       <c r="I214" s="14"/>
     </row>
-    <row r="215" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="215" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A215" s="14"/>
       <c r="B215" s="20"/>
       <c r="C215" s="20"/>
@@ -3215,7 +3211,7 @@
       <c r="H215" s="14"/>
       <c r="I215" s="14"/>
     </row>
-    <row r="216" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="216" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A216" s="14"/>
       <c r="B216" s="20"/>
       <c r="C216" s="20"/>
@@ -3226,7 +3222,7 @@
       <c r="H216" s="14"/>
       <c r="I216" s="14"/>
     </row>
-    <row r="217" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="217" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A217" s="14"/>
       <c r="B217" s="20"/>
       <c r="C217" s="20"/>
@@ -3237,7 +3233,7 @@
       <c r="H217" s="14"/>
       <c r="I217" s="14"/>
     </row>
-    <row r="218" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="218" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A218" s="14"/>
       <c r="B218" s="20"/>
       <c r="C218" s="20"/>
@@ -3248,7 +3244,7 @@
       <c r="H218" s="14"/>
       <c r="I218" s="14"/>
     </row>
-    <row r="219" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="219" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A219" s="14"/>
       <c r="B219" s="20"/>
       <c r="C219" s="20"/>
@@ -3259,7 +3255,7 @@
       <c r="H219" s="14"/>
       <c r="I219" s="14"/>
     </row>
-    <row r="220" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="220" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A220" s="14"/>
       <c r="B220" s="20"/>
       <c r="C220" s="20"/>
@@ -3270,7 +3266,7 @@
       <c r="H220" s="14"/>
       <c r="I220" s="14"/>
     </row>
-    <row r="221" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="221" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A221" s="14"/>
       <c r="B221" s="20"/>
       <c r="C221" s="20"/>
@@ -3281,7 +3277,7 @@
       <c r="H221" s="14"/>
       <c r="I221" s="14"/>
     </row>
-    <row r="222" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="222" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A222" s="14"/>
       <c r="B222" s="20"/>
       <c r="C222" s="20"/>
@@ -3292,7 +3288,7 @@
       <c r="H222" s="14"/>
       <c r="I222" s="14"/>
     </row>
-    <row r="223" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="223" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A223" s="14"/>
       <c r="B223" s="20"/>
       <c r="C223" s="20"/>
@@ -3303,7 +3299,7 @@
       <c r="H223" s="14"/>
       <c r="I223" s="14"/>
     </row>
-    <row r="224" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="224" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A224" s="14"/>
       <c r="B224" s="20"/>
       <c r="C224" s="20"/>
@@ -3314,7 +3310,7 @@
       <c r="H224" s="14"/>
       <c r="I224" s="14"/>
     </row>
-    <row r="225" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="225" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A225" s="14"/>
       <c r="B225" s="20"/>
       <c r="C225" s="20"/>
@@ -3325,7 +3321,7 @@
       <c r="H225" s="14"/>
       <c r="I225" s="14"/>
     </row>
-    <row r="226" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="226" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A226" s="14"/>
       <c r="B226" s="20"/>
       <c r="C226" s="20"/>
@@ -3336,7 +3332,7 @@
       <c r="H226" s="14"/>
       <c r="I226" s="14"/>
     </row>
-    <row r="227" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="227" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A227" s="14"/>
       <c r="B227" s="20"/>
       <c r="C227" s="20"/>
@@ -3347,7 +3343,7 @@
       <c r="H227" s="14"/>
       <c r="I227" s="14"/>
     </row>
-    <row r="228" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="228" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A228" s="14"/>
       <c r="B228" s="20"/>
       <c r="C228" s="20"/>
@@ -3358,7 +3354,7 @@
       <c r="H228" s="14"/>
       <c r="I228" s="14"/>
     </row>
-    <row r="229" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="229" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A229" s="14"/>
       <c r="B229" s="20"/>
       <c r="C229" s="20"/>
@@ -3369,7 +3365,7 @@
       <c r="H229" s="14"/>
       <c r="I229" s="14"/>
     </row>
-    <row r="230" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="230" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A230" s="14"/>
       <c r="B230" s="20"/>
       <c r="C230" s="20"/>
@@ -3380,7 +3376,7 @@
       <c r="H230" s="14"/>
       <c r="I230" s="14"/>
     </row>
-    <row r="231" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="231" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A231" s="14"/>
       <c r="B231" s="20"/>
       <c r="C231" s="20"/>
@@ -3391,7 +3387,7 @@
       <c r="H231" s="14"/>
       <c r="I231" s="14"/>
     </row>
-    <row r="232" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="232" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A232" s="14"/>
       <c r="B232" s="20"/>
       <c r="C232" s="20"/>
@@ -3402,7 +3398,7 @@
       <c r="H232" s="14"/>
       <c r="I232" s="14"/>
     </row>
-    <row r="233" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="233" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A233" s="14"/>
       <c r="B233" s="20"/>
       <c r="C233" s="20"/>
@@ -3413,7 +3409,7 @@
       <c r="H233" s="14"/>
       <c r="I233" s="14"/>
     </row>
-    <row r="234" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="234" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A234" s="14"/>
       <c r="B234" s="20"/>
       <c r="C234" s="20"/>
@@ -3424,7 +3420,7 @@
       <c r="H234" s="14"/>
       <c r="I234" s="14"/>
     </row>
-    <row r="235" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="235" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A235" s="14"/>
       <c r="B235" s="20"/>
       <c r="C235" s="20"/>
@@ -3435,7 +3431,7 @@
       <c r="H235" s="14"/>
       <c r="I235" s="14"/>
     </row>
-    <row r="236" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="236" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A236" s="14"/>
       <c r="B236" s="20"/>
       <c r="C236" s="20"/>
@@ -3446,7 +3442,7 @@
       <c r="H236" s="14"/>
       <c r="I236" s="14"/>
     </row>
-    <row r="237" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="237" spans="1:9" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A237" s="14"/>
       <c r="B237" s="20"/>
       <c r="C237" s="20"/>
@@ -3458,14 +3454,12 @@
       <c r="I237" s="14"/>
     </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="E26:H26"/>
+  <mergeCells count="7">
     <mergeCell ref="A2:A5"/>
     <mergeCell ref="B2:G3"/>
     <mergeCell ref="H2:H3"/>
     <mergeCell ref="I2:I3"/>
     <mergeCell ref="B4:G5"/>
-    <mergeCell ref="E25:H25"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="C6:I6"/>
   </mergeCells>

</xml_diff>